<commit_message>
Trien khai Web Dashboard tren GitHub Pages va xuat du lieu JSON
</commit_message>
<xml_diff>
--- a/data/Bao_Cao_Hoa_Don_Petrolimex.xlsx
+++ b/data/Bao_Cao_Hoa_Don_Petrolimex.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -869,6 +869,186 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:34:41.020000+00:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>2437203</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>35.006</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>25710</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>900000</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>900000</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>IY4WBHMAG*</t>
+        </is>
+      </c>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:22:49.934000+00:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>596130</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>51L-638.55</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Dầu Điêzen 0,001S Mức 5</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>50.425</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>30650</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>1545526</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>1545526</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>Quốc Lộ 51, Tổ 1, Ấp 1, Xã Phước Thái. Tp. Đồng Nai, VN</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>3Z4V2KNCG*</t>
+        </is>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId1"/>
@@ -877,6 +1057,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cap nhat hoa don Petrolimex 29/10/2026 10:47
</commit_message>
<xml_diff>
--- a/data/Bao_Cao_Hoa_Don_Petrolimex.xlsx
+++ b/data/Bao_Cao_Hoa_Don_Petrolimex.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1049,6 +1049,1446 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 06:58:05.848000+00:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2410305</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>25710</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>600000</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>B5VWBHMAG*</t>
+        </is>
+      </c>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:49:04.564000+00:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2398954</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>27520</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>1232346</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>1232346</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>6/5 Trần não, Phường An Khánh, TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>EJGEACMAG*</t>
+        </is>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:18:36.996000+00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>589682</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>51L-638.55</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Dầu Điêzen 0,001S Mức 5</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>33.123</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>30200</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>1000315</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>1000315</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>Quốc Lộ 51, Tổ 1, Ấp 1, Xã Phước Thái. Tp. Đồng Nai, VN</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>W5ZV2KNCG*</t>
+        </is>
+      </c>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:31:25.827000+00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2388772</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>25.44</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>27520</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>700110</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>700110</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>T7PWBHMAG*</t>
+        </is>
+      </c>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:46:55.878000+00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>583107</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 3</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>36.68</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>26720</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>980090</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>980090</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>1052, Đường QL 55,  Xã Long Điền, TP Hồ Chí Minh, Việt Nam</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>V7KMLSNCG*</t>
+        </is>
+      </c>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:43:36.032000+00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>583097</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>51L-638.55</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Dầu Điêzen 0,001S Mức 5</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>41.392</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>30200</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>1250038</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>1250038</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>Quốc Lộ 51, Tổ 1, Ấp 1, Xã Phước Thái. Tp. Đồng Nai, VN</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>JHXV2KNCG*</t>
+        </is>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:22:44.911000+00:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2362337</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>36.337</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>27520</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>YLIWBHMAG*</t>
+        </is>
+      </c>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 13:53:22.688000+00:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>577063</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>51L-638.55</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Dầu Điêzen 0,001S Mức 5</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>32.765</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>30520</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Quốc Lộ 51, Tổ 1, Ấp 1, Xã Phước Thái. Tp. Đồng Nai, VN</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>ZRUV2KNCG*</t>
+        </is>
+      </c>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:06:53.711000+00:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>2334702</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>46.56</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>29050</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>1352568</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>1352568</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>6/5 Trần não, Phường An Khánh, TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>ZIGDACMAG*</t>
+        </is>
+      </c>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 07:13:39.734000+00:00</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>2325107</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>27.54</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>29050</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>800000</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>800000</v>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>ZV7VBHMAG*</t>
+        </is>
+      </c>
+      <c r="S16" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 09:08:29.807000+00:00</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>2317548</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>37.87</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>29050</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>1100120</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>1100120</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>WR5VBHMAG*</t>
+        </is>
+      </c>
+      <c r="S17" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:24:55.430000+00:00</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>K26TXT</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>568861</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 3</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>30.091</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>28250</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>850071</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>850071</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH PETROLIMEX VŨNG TÀU - CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>1052, Đường QL 55,  Xã Long Điền, TP Hồ Chí Minh, Việt Nam</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>UAGMLSNCG*</t>
+        </is>
+      </c>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:21:32.508000+00:00</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>2295406</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>41.945</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>29050</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>1218502</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>1218502</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>6/5 Trần não, Phường An Khánh, TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>XRZCACMAG*</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:07:49.082000+00:00</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>2289616</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>51L-638.55</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Dầu Điêzen 0,001S Mức 5</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>40.173</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>31110</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>1249782</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>1249782</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>6/5 Trần não, Phường An Khánh, TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>A6WCACMAG*</t>
+        </is>
+      </c>
+      <c r="S20" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 10:11:34.291000+00:00</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>2278994</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>51K-229.32</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>32.302</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>28180</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>910270</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>910270</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>152 Nguyễn Khoái, Phường Vĩnh Hội, TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>CZFBANMAG*</t>
+        </is>
+      </c>
+      <c r="S21" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:31:59.044000+00:00</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>K26TAN</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>2250334</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>51M-159.48</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Xăng E10 RON 95 Mức 5</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>35.49</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>28180</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH MTV PETROLIMEX SÀI GÒN</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>178/6 Điện Biên Phủ,Phường Thạnh Mỹ Tây,TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>CÔNG TY CỔ PHẦN THÉP POVINA</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>WGKVBHMAG*</t>
+        </is>
+      </c>
+      <c r="S22" s="7" t="inlineStr">
+        <is>
+          <t>Xem PDF</t>
+        </is>
+      </c>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>Xem XML</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId1"/>
@@ -1061,6 +2501,38 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>